<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-01 Le petit pain chaud de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-01.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-01.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le petit pain fendu de Nino</t>
+          <t>Le petit pain chaud de Nino</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>vitrine givrée, puis boulangerie</t>
+          <t>rue froide, pavés, boulangerie, file près du bois, odeur de pain, four</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut le petit pain fendu derrière la vitre. Il dit bonjour, s'il te plaît, merci. Le sachet reste tiède.</t>
+          <t>Les pavés sonnent. Sur la pierre, un éclat de pavé luit. Nino veut le petit pain chaud maintenant. Il tend la main trop vite, sans le mot : la vitre arrête le doigt. Il refuse de foncer, dit s'il te plaît, obtient le sachet. Merci vécu. Un éclat de pavé reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Des fleurs de givre sont sur la vitrine. Un moineau se tient sur l'auvent. Une empreinte de farine reste sur le pas. Ça sent déjà le four, tout chaud. Tu sens, Nino ? Ça sent le beurre. La veste, un bouton de plus. Voilà. J'ai les joues froides. On marche. Tu restes près de nous. Nino pose le nez sur la vitre. Le givre fond un peu sous son souffle. Derrière, les pains sont alignés. Celui-là. Il a une fente. Le petit pain doré. On entre. La porte s'ouvre. L'air chaud fait comme un câlin. Une petite cloche fait ding. La farine est blanche sur le bois. En ce moment, Nino tient le manteau de maman. Le sol est tiède sous ses chaussures. La boulangère range encore des croûtes. Elle tourne le dos un moment. On attend un peu. Elle a les mains pleines. Nino regarde le petit pain fendu. Il avance le doigt vers la vitre du comptoir. Celui-là. Tu demandes, Nino. La boulangère se tourne. Un peu de farine est sur son tablier.</t>
+          <t>Les pavés sonnent sous les pas. Ils sont froids, un peu ronds. Sur la pierre, un éclat de pavé luit. Il brille, papa. Tu le vois, sur la rue ? Nino touche l'éclat de pavé, un instant. La pierre pique un peu le doigt. Elle est froide. La veste, un bouton de plus. Voilà. Un nuage blanc sort de la bouche. J'ai les joues froides. On marche. Tu restes près de nous ? Oui, maman. Une odeur de pain arrive. Elle vient du four. Ça sent le four ! Tu sens, Nino ? Oui. La porte de bois attend. Une petite cloche fait ding. L'air chaud touche les joues. Une file avance près du bois. On reste dans la file. Des manteaux se touchent dans la file. Ça sent le beurre, un peu chaud. Je le veux, maintenant. En ce moment, Nino serre le manteau. Le sol est tiède sous ses chaussures. Le bois du comptoir est lisse. Le four est là. Il chauffe derrière le mur. Une lueur orange tient derrière le verre. Nino se dresse sur les pointes. Un petit pain doré attend derrière la vitre. Celui-là ! Nino tend la main trop vite. Le doigt tape la vitre. Oh. Le pain reste derrière le verre. La file n'a pas bougé. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le pain est derrière le verre. Tu le vois, Nino ? Les épaules de Nino tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Des fleurs de givre sont sur la vitrine. Un moineau se tient sur l'auvent. Une empreinte de farine reste sur le pas. Ça sent déjà le four, tout chaud. Tu sens, Nino ? Ça sent le beurre. La veste, un bouton de plus. Voilà. J'ai les joues froides. On marche. Tu restes près de nous. Nino pose le nez sur la vitre. Le givre fond un peu sous son souffle. Derrière, les pains sont alignés. Celui-là. Il a une fente. Le petit pain doré. On entre. La porte s'ouvre. L'air chaud fait comme un câlin. Une petite cloche fait ding. La farine est blanche sur le bois. En ce moment, Nino tient le manteau de maman. Le sol est tiède sous ses chaussures. La boulangère range encore des croûtes. Elle tourne le dos un moment. On attend un peu. Elle a les mains pleines. Nino regarde le petit pain fendu. Il avance le doigt vers la vitre du comptoir. Celui-là. Tu demandes, Nino. La boulangère se tourne. Un peu de farine est sur son tablier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les pavés sonnent sous les pas. Ils sont froids, un peu ronds. Sur la pierre, un &lt;emphasis level="moderate"&gt;éclat de pavé&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur la rue ? Nino touche l'éclat de pavé, un instant. La pierre pique un peu le doigt. Elle est froide. La veste, un bouton de plus. Voilà. Un nuage blanc sort de la bouche. J'ai les joues froides. On marche. Tu restes près de nous ? Oui, maman. Une odeur de pain arrive. Elle vient du four. Ça sent le four ! Tu sens, Nino ? Oui. La porte de bois attend. Une petite cloche fait ding. L'air chaud touche les joues. Une file avance près du bois. On reste dans la file. Des manteaux se touchent dans la file. Ça sent le beurre, un peu chaud. Je le veux, maintenant. En ce moment, Nino serre le manteau. Le sol est tiède sous ses chaussures. Le bois du comptoir est lisse. Le four est là. Il chauffe derrière le mur. Une lueur orange tient derrière le verre. Nino se dresse sur les pointes. Un petit pain doré attend derrière la vitre. Celui-là ! Nino tend la main trop vite. Le doigt tape la vitre. Oh. Le pain reste derrière le verre. La file n'a pas bougé. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le pain est derrière le verre. Tu le vois, Nino ? Les épaules de Nino tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom marche avec maman. Ils vont à la boulangerie. La cloche fait ding. La boulangère sourit. Tom dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Maman dit : bonjour. Tom pointe un petit pain. Il dit : s'il te plaît. La boulangère tend le pain. Tom dit : merci. Maman dit : merci. Tom tient le pain chaud. Ça sent bon. Maman serre sa main. Tom répète : bonjour. S'il te plaît. Merci. Les trois mots sont là.&lt;/slow&gt; [pause]</t>
+          <t>Les pavés sonnent sous les pas. Ils sont froids, un peu ronds. Sur la pierre, un &lt;emphasis&gt;éclat de pavé&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur la rue ? Nino touche l'éclat de pavé, un instant. La pierre pique un peu le doigt. Elle est froide. La veste, un bouton de plus. Voilà. Un nuage blanc sort de la bouche. J'ai les joues froides. On marche. Tu restes près de nous ? Oui, maman. Une odeur de pain arrive. Elle vient du four. Ça sent le four ! Tu sens, Nino ? Oui. La porte de bois attend. Une petite cloche fait ding. L'air chaud touche les joues. Une file avance près du bois. On reste dans la file. Des manteaux se touchent dans la file. Ça sent le beurre, un peu chaud. Je le veux, maintenant. En ce moment, Nino serre le manteau. Le sol est tiède sous ses chaussures. Le bois du comptoir est lisse. Le four est là. Il chauffe derrière le mur. Une lueur orange tient derrière le verre. Nino se dresse sur les pointes. Un petit pain doré attend derrière la vitre. Celui-là ! Nino tend la main trop vite. Le doigt tape la vitre. Oh. Le pain reste derrière le verre. La file n'a pas bougé. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le pain est derrière le verre. Tu le vois, Nino ? Les épaules de Nino tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de pavé</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,50 +1324,70 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_pain_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Des fleurs de givre sont sur la vitrine.
-narrateur|Un moineau se tient sur l'auvent.
-narrateur|Une empreinte de farine reste sur le pas.
-narrateur|Ça sent déjà le four, tout chaud.
-maman|Tu sens, Nino ?
-maman|Ça sent le beurre.
-papa|La veste, un bouton de plus.
+          <t>narrateur|Les pavés sonnent sous les pas.
+narrateur|Ils sont froids, un peu ronds.
+narrateur|Sur la pierre, un éclat de pavé luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur la rue ?
+narrateur|Nino touche l'éclat de pavé, un instant.
+narrateur|La pierre pique un peu le doigt.
+enfant-m|Elle est froide.
+maman|La veste, un bouton de plus.
 papa|Voilà.
+narrateur|Un nuage blanc sort de la bouche.
 enfant-m|J'ai les joues froides.
 papa|On marche.
-papa|Tu restes près de nous.
-narrateur|Nino pose le nez sur la vitre.
-narrateur|Le givre fond un peu sous son souffle.
-narrateur|Derrière, les pains sont alignés.
-enfant-m|Celui-là.
-enfant-m|Il a une fente.
-maman|Le petit pain doré.
-papa|On entre.
-narrateur|La porte s'ouvre.
-narrateur|L'air chaud fait comme un câlin.
+maman|Tu restes près de nous ?
+enfant-m|Oui, maman.
+narrateur|Une odeur de pain arrive.
+narrateur|Elle vient du four.
+enfant-m|Ça sent le four !
+maman|Tu sens, Nino ?
+enfant-m|Oui.
+narrateur|La porte de bois attend.
 narrateur|Une petite cloche fait ding.
-narrateur|La farine est blanche sur le bois.
-narrateur|En ce moment, Nino tient le manteau de maman.
+narrateur|L'air chaud touche les joues.
+narrateur|Une file avance près du bois.
+papa|On reste dans la file.
+narrateur|Des manteaux se touchent dans la file.
+narrateur|Ça sent le beurre, un peu chaud.
+enfant-m|Je le veux, maintenant.
+narrateur|En ce moment, Nino serre le manteau.
 narrateur|Le sol est tiède sous ses chaussures.
-narrateur|La boulangère range encore des croûtes.
-narrateur|Elle tourne le dos un moment.
-maman|On attend un peu.
-papa|Elle a les mains pleines.
-narrateur|Nino regarde le petit pain fendu.
-narrateur|Il avance le doigt vers la vitre du comptoir.
-enfant-m|Celui-là.
-maman|Tu demandes, Nino.
-narrateur|La boulangère se tourne.
-narrateur|Un peu de farine est sur son tablier.</t>
+narrateur|Le bois du comptoir est lisse.
+enfant-m|Le four est là.
+maman|Il chauffe derrière le mur.
+narrateur|Une lueur orange tient derrière le verre.
+narrateur|Nino se dresse sur les pointes.
+narrateur|Un petit pain doré attend derrière la vitre.
+enfant-m|Celui-là !
+narrateur|Nino tend la main trop vite.
+narrateur|Le doigt tape la vitre.
+enfant-m|Oh.
+narrateur|Le pain reste derrière le verre.
+narrateur|La file n'a pas bougé.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Je le prends !
+maman|Le pain est derrière le verre.
+papa|Tu le vois, Nino ?
+narrateur|Les épaules de Nino tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>cloche,papier</t>
+          <t>cloche,pas</t>
         </is>
       </c>
     </row>
@@ -1399,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino veut le pain. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino veut le &lt;emphasis level="moderate"&gt;pain&lt;/emphasis&gt;. Que dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom veut le pain. Que dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino veut le &lt;emphasis&gt;pain&lt;/emphasis&gt;. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1467,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1475,10 +1495,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1493,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>pain</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1529,13 +1553,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1545,7 +1569,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_dit_s_il_te_plait; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1578,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Bonjour. Le petit pain, s'il te plaît. Celui avec la fente. La boulangère pose le pain dans un sachet. Le papier fait un bruit doux. Le pain est encore chaud. Merci. Merci. Tu as dit s'il te plaît. Nino tient le sachet contre son manteau. Ça sent le beurre et le four. Tu as les mains au chaud ? Oui. Le pain est chaud. Le bois du comptoir est lisse. Nino pose une main sur le sachet. Le papier est un peu rêche. On dit au revoir, maintenant. Au revoir. Au revoir. La cloche fait ding, encore. L'air froid revient sur les joues.</t>
+          <t>Nino avance trop vite vers le bois. Celui-là, maintenant ! Sa voix se mélange à la file. Oh. Le petit pain reste derrière la vitre. Il refuse de foncer. Nino referme la main. Il écoute la cloche, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Nino pose un pied sur le pas. Le bois est tiède, un peu lisse. Celui-là. S'il te plaît. Derrière le bois, une main se tend. Le papier enveloppe le pain. Le sachet est chaud contre le manteau. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le four. Le pain est à moi. Il est dans tes mains. Nino pose une main sur le sachet. Le papier est un peu rêche. La cloche se tait.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Bonjour. Le petit pain, s'il te plaît. Celui avec la fente. La boulangère pose le pain dans un sachet. Le papier fait un bruit doux. Le pain est encore chaud. Merci. Merci. Tu as dit s'il te plaît. Nino tient le sachet contre son manteau. Ça sent le beurre et le four. Tu as les mains au chaud ? Oui. Le pain est chaud. Le bois du comptoir est lisse. Nino pose une main sur le sachet. Le papier est un peu rêche. On dit au revoir, maintenant. Au revoir. Au revoir. La cloche fait ding, encore. L'air froid revient sur les joues.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino avance trop vite vers le bois. Celui-là, maintenant ! Sa voix se mélange à la file. Oh. Le petit pain reste derrière la vitre. Il refuse de foncer. Nino referme la main. Il écoute la cloche, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Nino pose un pied sur le pas. Le bois est tiède, un peu lisse. Celui-là. S'il te plaît. Derrière le bois, une main se tend. Le papier enveloppe le pain. Le sachet est chaud contre le manteau. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le four. Le pain est à moi. Il est dans tes mains. Nino pose une main sur le sachet. Le papier est un peu rêche. La cloche se tait.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Il a dit s'il te plaît. Il a dit merci. Maman est là.&lt;/slow&gt; [pause]</t>
+          <t>Nino avance trop vite vers le bois. Celui-là, maintenant ! Sa voix se mélange à la file. Oh. Le petit pain reste derrière la vitre. Il refuse de foncer. Nino referme la main. Il écoute la cloche, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Nino pose un pied sur le pas. Le bois est tiède, un peu lisse. Celui-là. S'il te plaît. Derrière le bois, une main se tend. Le papier enveloppe le pain. Le sachet est chaud contre le manteau. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le four. Le pain est à moi. Il est dans tes mains. Nino pose une main sur le sachet. Le papier est un peu rêche. La cloche se tait. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1635,18 +1659,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,20 +1703,20 @@
         <v>450</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1701,10 +1725,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1713,44 +1737,49 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_vitre_echoue_le_mot_ouvre; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Bonjour.
-maman|Bonjour.
-papa|Bonjour.
-enfant-m|Le petit pain, s'il te plaît.
-enfant-m|Celui avec la fente.
-narrateur|La boulangère pose le pain dans un sachet.
-narrateur|Le papier fait un bruit doux.
-narrateur|Le pain est encore chaud.
-enfant-m|Merci.
-papa|Merci.
-maman|Tu as dit s'il te plaît.
-narrateur|Nino tient le sachet contre son manteau.
+          <t>narrateur|Nino avance trop vite vers le bois.
+enfant-m|Celui-là, maintenant !
+narrateur|Sa voix se mélange à la file.
+enfant-m|Oh.
+narrateur|Le petit pain reste derrière la vitre.
+narrateur|Il refuse de foncer.
+narrateur|Nino referme la main.
+narrateur|Il écoute la cloche, un instant.
+papa|Tu veux venir près du bois ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Nino pose un pied sur le pas.
+narrateur|Le bois est tiède, un peu lisse.
+enfant-m|Celui-là.
+enfant-m|S'il te plaît.
+narrateur|Derrière le bois, une main se tend.
+narrateur|Le papier enveloppe le pain.
+narrateur|Le sachet est chaud contre le manteau.
+papa|Merci, Nino.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-m|Un peu, maman.
 narrateur|Ça sent le beurre et le four.
-maman|Tu as les mains au chaud ?
-enfant-m|Oui.
-enfant-m|Le pain est chaud.
-narrateur|Le bois du comptoir est lisse.
+enfant-m|Le pain est à moi.
+maman|Il est dans tes mains.
 narrateur|Nino pose une main sur le sachet.
 narrateur|Le papier est un peu rêche.
-papa|On dit au revoir, maintenant.
-enfant-m|Au revoir.
-maman|Au revoir.
-narrateur|La cloche fait ding, encore.
-narrateur|L'air froid revient sur les joues.</t>
+narrateur|La cloche se tait.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>papier</t>
+          <t>papier,cloche</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1806,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sur le chemin, le sachet reste tiède. Tu veux un petit bout, Nino ? Oui. S'il te plaît. Maman déchire un bout de croûte. Nino croque. C'est chaud. C'est bon. La fente est encore là. Oui. Et merci, maintenant ? Merci, maman. Merci, Nino. Le moineau n'est plus sur l'auvent. Tu tiens le sachet des deux mains ? Oui, papa. Tu marches près de nous. Les fleurs de givre ont fondu. La maison sent déjà le pain. Nino pose le sachet sur la table. Il est encore tiède. On le garde pour plus tard. Un petit bout, déjà. Oui. C'était bon.</t>
+          <t>Nino tire le sachet trop vite. Je le mange, d'un coup ! Le papier glisse entre les doigts. Le pain penche vers le sol. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Nino observe le pas, écoute la rue. Sur la pierre, un éclat de pavé luit. Là, près de la porte. Nino tient le sachet des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air froid revient sur les joues. Nino serre le sachet contre lui. Il reste chaud. On marche. Le sachet penche, puis se cale. Je le tiens. On avance. Nino passe le pas de bois. Le bois craque, un peu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sur le chemin, le sachet reste tiède. Tu veux un petit bout, Nino ? Oui. S'il te plaît. Maman déchire un bout de croûte. Nino croque. C'est chaud. C'est bon. La fente est encore là. Oui. Et merci, maintenant ? Merci, maman. Merci, Nino. Le moineau n'est plus sur l'auvent. Tu tiens le sachet des deux mains ? Oui, papa. Tu marches près de nous. Les fleurs de givre ont fondu. La maison sent déjà le pain. Nino pose le sachet sur la table. Il est encore tiède. On le garde pour plus tard. Un petit bout, déjà. Oui. C'était bon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino tire le sachet trop vite. Je le mange, d'un coup ! Le papier glisse entre les doigts. Le pain penche vers le sol. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Nino observe le pas, écoute la rue. Sur la pierre, un &lt;emphasis level="moderate"&gt;éclat de pavé&lt;/emphasis&gt; luit. Là, près de la porte. Nino tient le sachet des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air froid revient sur les joues. Nino serre le sachet contre lui. Il reste chaud. On marche. Le sachet penche, puis se cale. Je le tiens. On avance. Nino passe le pas de bois. Le bois craque, un peu.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom croque un bout de pain. Maman sourit.&lt;/slow&gt; [pause]</t>
+          <t>Nino tire le sachet trop vite. Je le mange, d'un coup ! Le papier glisse entre les doigts. Le pain penche vers le sol. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Nino observe le pas, écoute la rue. Sur la pierre, un &lt;emphasis&gt;éclat de pavé&lt;/emphasis&gt; luit. Là, près de la porte. Nino tient le sachet des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air froid revient sur les joues. Nino serre le sachet contre lui. Il reste chaud. On marche. Le sachet penche, puis se cale. Je le tiens. On avance. Nino passe le pas de bois. Le bois craque, un peu. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,18 +1863,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1866,28 +1895,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pavé</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,10 +1929,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,36 +1941,45 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sur le chemin, le sachet reste tiède.
-maman|Tu veux un petit bout, Nino ?
-enfant-m|Oui.
-enfant-m|S'il te plaît.
-narrateur|Maman déchire un bout de croûte.
-narrateur|Nino croque.
-enfant-m|C'est chaud.
-enfant-m|C'est bon.
-papa|La fente est encore là.
-enfant-m|Oui.
-maman|Et merci, maintenant ?
-enfant-m|Merci, maman.
-papa|Merci, Nino.
-narrateur|Le moineau n'est plus sur l'auvent.
-papa|Tu tiens le sachet des deux mains ?
+          <t>narrateur|Nino tire le sachet trop vite.
+enfant-m|Je le mange, d'un coup !
+narrateur|Le papier glisse entre les doigts.
+narrateur|Le pain penche vers le sol.
+enfant-m|Oh.
+narrateur|Nino avance les mains.
+narrateur|Puis il s'arrête net.
+enfant-m|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Nino observe le pas, écoute la rue.
+narrateur|Sur la pierre, un éclat de pavé luit.
+enfant-m|Là, près de la porte.
+narrateur|Nino tient le sachet des deux mains.
+narrateur|Le papier est rêche, un peu chaud.
+enfant-m|Il est chaud, papa.
+papa|Tu le portes jusqu'à la rue ?
 enfant-m|Oui, papa.
-maman|Tu marches près de nous.
-narrateur|Les fleurs de givre ont fondu.
-narrateur|La maison sent déjà le pain.
-narrateur|Nino pose le sachet sur la table.
-enfant-m|Il est encore tiède.
-maman|On le garde pour plus tard.
-papa|Un petit bout, déjà.
-enfant-m|Oui.
-enfant-m|C'était bon.</t>
+maman|On sort ?
+enfant-m|Oui, maman.
+narrateur|La porte s'ouvre.
+narrateur|La cloche fait ding.
+narrateur|L'air froid revient sur les joues.
+narrateur|Nino serre le sachet contre lui.
+enfant-m|Il reste chaud.
+papa|On marche.
+narrateur|Le sachet penche, puis se cale.
+enfant-m|Je le tiens.
+maman|On avance.
+narrateur|Nino passe le pas de bois.
+narrateur|Le bois craque, un peu.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1969,17 +2011,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le sachet repose sur la table. Il reste un bout, encore tiède. Bonne journée, mon grand. Le petit pain avait une fente.</t>
+          <t>Le pavé brillait, papa. Tu le vois, comme dans la rue ? Oui, sur la pierre. Nino pose le sachet contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Nino respire, plus large. On rentre ? Oui. Les joues de Nino se réchauffent. Le sachet reste tiède sous la main. Un éclat de pavé reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le sachet repose sur la table. Il reste un bout, encore tiède. Bonne journée, mon grand. Le petit pain avait une fente.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le pavé brillait, papa. Tu le vois, comme dans la rue ? Oui, sur la pierre. Nino pose le sachet contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Nino respire, plus large. On rentre ? Oui. Les joues de Nino se réchauffent. Le sachet reste tiède sous la main. Un &lt;emphasis level="moderate"&gt;éclat de pavé&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le pavé brillait, papa. Tu le vois, comme dans la rue ? Oui, sur la pierre. Nino pose le sachet contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Nino respire, plus large. On rentre ? Oui. Les joues de Nino se réchauffent. Le sachet reste tiède sous la main. Un &lt;emphasis&gt;éclat de pavé&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2026,7 +2068,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2034,10 +2076,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2046,12 +2088,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2060,17 +2102,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pavé</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2079,11 +2125,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2092,27 +2138,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le sachet repose sur la table.
-narrateur|Il reste un bout, encore tiède.
-maman|Bonne journée, mon grand.
-papa|Le petit pain avait une fente.</t>
+          <t>enfant-m|Le pavé brillait, papa.
+papa|Tu le vois, comme dans la rue ?
+enfant-m|Oui, sur la pierre.
+narrateur|Nino pose le sachet contre le manteau.
+maman|On le garde au chaud ?
+enfant-m|Oui, maman.
+enfant-m|Le four sentait bon.
+maman|Il est contre toi.
+narrateur|Une vapeur monte du papier.
+narrateur|Nino respire, plus large.
+papa|On rentre ?
+enfant-m|Oui.
+narrateur|Les joues de Nino se réchauffent.
+narrateur|Le sachet reste tiède sous la main.
+narrateur|Un éclat de pavé reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pas</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2284,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>